<commit_message>
Update inventory management system
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,34 +440,66 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pen</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="C2" t="n">
+        <v>36000</v>
+      </c>
+      <c r="D2" t="n">
         <v>10</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>35000</v>
+        <v>55000</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>